<commit_message>
Add TF (Trust Flow) column to medical/health selection sheets
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTSVFSSCJZESeLBYWra4gT
</commit_message>
<xml_diff>
--- a/BlueGoatCyber_Medical_Health_Additions.xlsx
+++ b/BlueGoatCyber_Medical_Health_Additions.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Medical-Health additions'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Your selection (11)'!$A$1:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Medical-Health additions'!$A$1:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Your selection (11)'!$A$1:$I$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -563,17 +563,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -597,22 +598,27 @@
           <t>Semrush AS</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>TF</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>US Organic Traffic</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total Traffic</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Price ($)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -635,16 +641,19 @@
       <c r="D2" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E2" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F2" s="8" t="n">
         <v>74419</v>
       </c>
-      <c r="F2" s="9" t="n">
+      <c r="G2" s="9" t="n">
         <v>71655</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="H2" s="10" t="n">
         <v>160</v>
       </c>
-      <c r="H2" s="11" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>US physician directory &amp; medical content (best pick)</t>
         </is>
@@ -667,16 +676,19 @@
       <c r="D3" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="F3" s="8" t="n">
         <v>53568</v>
       </c>
-      <c r="F3" s="15" t="n">
+      <c r="G3" s="15" t="n">
         <v>98711</v>
       </c>
-      <c r="G3" s="16" t="n">
+      <c r="H3" s="16" t="n">
         <v>197</v>
       </c>
-      <c r="H3" s="17" t="inlineStr">
+      <c r="I3" s="17" t="inlineStr">
         <is>
           <t>Anatomy / manual-therapy education (US)</t>
         </is>
@@ -699,16 +711,19 @@
       <c r="D4" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="F4" s="8" t="n">
         <v>26588</v>
       </c>
-      <c r="F4" s="9" t="n">
+      <c r="G4" s="9" t="n">
         <v>36592</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="H4" s="10" t="n">
         <v>200</v>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Psychology &amp; mental-health publication (US)</t>
         </is>
@@ -731,16 +746,19 @@
       <c r="D5" s="7" t="n">
         <v>38</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F5" s="8" t="n">
         <v>16487</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="G5" s="15" t="n">
         <v>14063</v>
       </c>
-      <c r="G5" s="16" t="n">
+      <c r="H5" s="16" t="n">
         <v>200</v>
       </c>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>US mental-health / counseling practice</t>
         </is>
@@ -763,16 +781,19 @@
       <c r="D6" s="7" t="n">
         <v>37</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="F6" s="8" t="n">
         <v>14113</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="G6" s="9" t="n">
         <v>19633</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="H6" s="10" t="n">
         <v>160</v>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>Wellness &amp; mindful-living (US)</t>
         </is>
@@ -795,16 +816,19 @@
       <c r="D7" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F7" s="8" t="n">
         <v>13891</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="G7" s="15" t="n">
         <v>24093</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="H7" s="16" t="n">
         <v>250</v>
       </c>
-      <c r="H7" s="17" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>Child health &amp; parenting nonprofit (.org)</t>
         </is>
@@ -827,16 +851,19 @@
       <c r="D8" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="F8" s="8" t="n">
         <v>13048</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="G8" s="9" t="n">
         <v>30953</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="H8" s="10" t="n">
         <v>200</v>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>Women's hormone-health nonprofit (.org)</t>
         </is>
@@ -859,16 +886,19 @@
       <c r="D9" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="F9" s="8" t="n">
         <v>12920</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="G9" s="15" t="n">
         <v>14167</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="H9" s="16" t="n">
         <v>140</v>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>Senior living / assisted care (US)</t>
         </is>
@@ -891,16 +921,19 @@
       <c r="D10" s="7" t="n">
         <v>39</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="F10" s="8" t="n">
         <v>9268</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="G10" s="9" t="n">
         <v>18836</v>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="H10" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>Pet health-tech / wearable device (US)</t>
         </is>
@@ -923,16 +956,19 @@
       <c r="D11" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="F11" s="8" t="n">
         <v>6046</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="G11" s="15" t="n">
         <v>14914</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="H11" s="16" t="n">
         <v>170</v>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>Dental resources / oral health (.org)</t>
         </is>
@@ -955,16 +991,19 @@
       <c r="D12" s="7" t="n">
         <v>38</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="F12" s="8" t="n">
         <v>5182</v>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="G12" s="9" t="n">
         <v>15120</v>
       </c>
-      <c r="G12" s="10" t="n">
+      <c r="H12" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>US dental professionals community</t>
         </is>
@@ -987,23 +1026,26 @@
       <c r="D13" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="F13" s="8" t="n">
         <v>2177</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="G13" s="15" t="n">
         <v>4159</v>
       </c>
-      <c r="G13" s="16" t="n">
+      <c r="H13" s="16" t="n">
         <v>230</v>
       </c>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="I13" s="17" t="inlineStr">
         <is>
           <t>Medical &amp; science news (lower traffic)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:I13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1014,17 +1056,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1048,22 +1091,27 @@
           <t>Semrush AS</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>TF</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>US Organic Traffic</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total Traffic</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Price ($)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1086,16 +1134,19 @@
       <c r="D2" s="7" t="n">
         <v>52</v>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E2" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="F2" s="8" t="n">
         <v>36081</v>
       </c>
-      <c r="F2" s="9" t="n">
+      <c r="G2" s="9" t="n">
         <v>3645809</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="H2" s="10" t="n">
         <v>250</v>
       </c>
-      <c r="H2" s="11" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>Tech/how-to (India+US audience)</t>
         </is>
@@ -1118,16 +1169,19 @@
       <c r="D3" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F3" s="8" t="n">
         <v>87620</v>
       </c>
-      <c r="F3" s="15" t="n">
+      <c r="G3" s="15" t="n">
         <v>537885</v>
       </c>
-      <c r="G3" s="16" t="n">
+      <c r="H3" s="16" t="n">
         <v>250</v>
       </c>
-      <c r="H3" s="17" t="inlineStr">
+      <c r="I3" s="17" t="inlineStr">
         <is>
           <t>Business &amp; tech opinion</t>
         </is>
@@ -1150,16 +1204,19 @@
       <c r="D4" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="F4" s="8" t="n">
         <v>23693</v>
       </c>
-      <c r="F4" s="9" t="n">
+      <c r="G4" s="9" t="n">
         <v>274538</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="H4" s="10" t="n">
         <v>61</v>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Collaborative docs; dev/security</t>
         </is>
@@ -1182,16 +1239,19 @@
       <c r="D5" s="7" t="n">
         <v>47</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="F5" s="8" t="n">
         <v>59331</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="G5" s="15" t="n">
         <v>265910</v>
       </c>
-      <c r="G5" s="16" t="n">
+      <c r="H5" s="16" t="n">
         <v>190</v>
       </c>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>ITSM / IT management blog</t>
         </is>
@@ -1214,16 +1274,19 @@
       <c r="D6" s="7" t="n">
         <v>49</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="F6" s="8" t="n">
         <v>7742</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="G6" s="9" t="n">
         <v>112033</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="H6" s="10" t="n">
         <v>250</v>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>AI &amp; data-science publication</t>
         </is>
@@ -1246,16 +1309,19 @@
       <c r="D7" s="7" t="n">
         <v>43</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="F7" s="8" t="n">
         <v>27212</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="G7" s="15" t="n">
         <v>41894</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="H7" s="16" t="n">
         <v>250</v>
       </c>
-      <c r="H7" s="17" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>Gadgets &amp; tech reviews</t>
         </is>
@@ -1278,16 +1344,19 @@
       <c r="D8" s="7" t="n">
         <v>39</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="F8" s="8" t="n">
         <v>3433</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="G8" s="9" t="n">
         <v>37120</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="H8" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>Tech news &amp; reviews</t>
         </is>
@@ -1310,16 +1379,19 @@
       <c r="D9" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="F9" s="8" t="n">
         <v>22712</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="G9" s="15" t="n">
         <v>34365</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="H9" s="16" t="n">
         <v>150</v>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>Home business &amp; entrepreneurship</t>
         </is>
@@ -1342,16 +1414,19 @@
       <c r="D10" s="7" t="n">
         <v>43</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="F10" s="8" t="n">
         <v>15922</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="G10" s="9" t="n">
         <v>27225</v>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="H10" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>Market research &amp; business</t>
         </is>
@@ -1374,16 +1449,19 @@
       <c r="D11" s="7" t="n">
         <v>37</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="F11" s="8" t="n">
         <v>3018</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="G11" s="15" t="n">
         <v>11962</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="H11" s="16" t="n">
         <v>170</v>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>Business &amp; technology magazine</t>
         </is>
@@ -1406,23 +1484,26 @@
       <c r="D12" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F12" s="8" t="n">
         <v>2420</v>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="G12" s="9" t="n">
         <v>5584</v>
       </c>
-      <c r="G12" s="10" t="n">
+      <c r="H12" s="10" t="n">
         <v>235</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>Cybersecurity directory &amp; news</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H12"/>
+  <autoFilter ref="A1:I12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1433,7 +1514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1452,76 +1533,38 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tab 'Medical-Health additions': 12 medical/health sites found per your request.</t>
+          <t>Metric key: Semrush AS = Authority Score (live) | TF = Trust Flow (Majestic, from inventory) |</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - All verified live on Semrush (Authority Score + US organic traffic).</t>
+          <t>US Organic Traffic = live Semrush (us DB) | Total Traffic = inventory global estimate.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - All US-focused, &lt;= $250, and NOT already used (checked vs Ahrefs + Semrush referring</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">    domains and your May-Aug '25 built list).</t>
+          <t>Medical-Health additions: 12 sites, all US-focused, &lt;= $250, and NOT already used</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - findatopdoc.com is the standout (AS 50, US 74k, physician directory).</t>
+          <t>(checked vs Ahrefs + Semrush referring domains and your May-Aug '25 built list).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - medicalnewsbulletin.com kept as optional (low US traffic ~2.2k).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Excluded health sites that were already used/built or off-target: yourhealthmagazine.net,</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>plasticsurgerykey.com, musculoskeletalkey.com, radiologykey.com (PBN network), medigy,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>credihealth, rightpatient, openmedscience, seniorliving, briancolemd, healsecurity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Tab 'Your selection (11)': the 11 you kept, with live Semrush AS + US traffic for reference.</t>
+          <t>findatopdoc.com is the standout (AS 50, TF 30, US 74k). medicalnewsbulletin optional (low traffic).</t>
         </is>
       </c>
     </row>

</xml_diff>